<commit_message>
data: update 2026-05-27 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/daily_logs/daily_2026-05-27.xlsx
+++ b/daily_logs/daily_2026-05-27.xlsx
@@ -18,9 +18,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -236,7 +235,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -275,7 +274,8 @@
     <xf numFmtId="58" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -674,7 +674,7 @@
           <t>Date</t>
         </is>
       </c>
-      <c r="B4" s="30" t="n">
+      <c r="B4" s="31" t="n">
         <v>46169</v>
       </c>
       <c r="C4" s="28" t="n"/>
@@ -2916,6 +2916,10 @@
         <is>
           <t>HY OAS 20dd=10.0bp [OK]
 HY OAS 5dd=9.0bp
+HYG 5d=0.8% [OK]
+HYG DD%=None% max drawdown
+FXY 5d=-0.3% [OK]
+SPY vs 200MA: above ($SPY=750.5900268554688, 200MA=676.9)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>